<commit_message>
Modifying the script to be able to read a destination from servers as well.
</commit_message>
<xml_diff>
--- a/Natus_filenames_for_RBD.xlsx
+++ b/Natus_filenames_for_RBD.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CEAMS\Projet du Soraya\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ceams_dev\projects\snooz\RenameNatus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{177345EF-CA19-4D66-BCF1-1625DF3C4938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB08D66-CE3F-4AF8-B180-06626B7DF455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1980" yWindow="1485" windowWidth="21600" windowHeight="11235" xr2:uid="{5AE431A0-7764-4F08-9AC7-CCB95F65E296}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5AE431A0-7764-4F08-9AC7-CCB95F65E296}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Code</t>
   </si>
@@ -100,12 +100,6 @@
   </si>
   <si>
     <t>Xxxxxxx~ Xxxx_58e057ec-d3fc-4991-89d5-54a979092bca</t>
-  </si>
-  <si>
-    <t>RT</t>
-  </si>
-  <si>
-    <t>COV-024~ COVID_938e31ce-88c4-487f-b02b-aba22c66c83f</t>
   </si>
 </sst>
 </file>
@@ -495,7 +489,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEE0E6B9-2D35-4ED7-AF40-2B077617D2BB}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="22.75" customWidth="1"/>
   </cols>
@@ -611,15 +605,7 @@
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="3">
-        <v>46301</v>
-      </c>
-      <c r="C11" t="s">
-        <v>22</v>
-      </c>
+      <c r="B11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>